<commit_message>
feat: implement Sumber Dana Tambahan tab and CSP fix
- Add SumberDanaSekolah model + migration
- ArkasImportService: import sheet Ref_Sumber_Dana defensively
- RkasController::index: tambahan list + filter ?sumber_nama
- View rkas.index: chip nama sumber + CTA Tarik/Perbarui Data
- Fixture arkas-mini: add Ref_Sumber_Dana sheet + regenerate
- SumberDanaTambahanTest: import, filter, CTA scenarios
- AsetHalamanTest: fake dev server probe + restore public/hot
- CSP: public/hot → http://localhost:5173 (valid for Chromium)
- Pint format check passed

Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/tests/Fixtures/arkas-asing.xlsx
+++ b/tests/Fixtures/arkas-asing.xlsx
@@ -12,14 +12,15 @@
     <sheet name="Penjab" sheetId="3" r:id="rId6"/>
     <sheet name="Salur" sheetId="4" r:id="rId7"/>
     <sheet name="Ref_Rekening" sheetId="5" r:id="rId8"/>
-    <sheet name="Aktivasi_BKU" sheetId="6" r:id="rId9"/>
-    <sheet name="PTK" sheetId="7" r:id="rId10"/>
-    <sheet name="RAPBS" sheetId="8" r:id="rId11"/>
-    <sheet name="Ref_Kode" sheetId="9" r:id="rId12"/>
-    <sheet name="RAPBS_Periode" sheetId="10" r:id="rId13"/>
-    <sheet name="KAS_Umum" sheetId="11" r:id="rId14"/>
-    <sheet name="Nota" sheetId="12" r:id="rId15"/>
-    <sheet name="Pajak_NTPN" sheetId="13" r:id="rId16"/>
+    <sheet name="Ref_Sumber_Dana" sheetId="6" r:id="rId9"/>
+    <sheet name="Aktivasi_BKU" sheetId="7" r:id="rId10"/>
+    <sheet name="PTK" sheetId="8" r:id="rId11"/>
+    <sheet name="RAPBS" sheetId="9" r:id="rId12"/>
+    <sheet name="Ref_Kode" sheetId="10" r:id="rId13"/>
+    <sheet name="RAPBS_Periode" sheetId="11" r:id="rId14"/>
+    <sheet name="KAS_Umum" sheetId="12" r:id="rId15"/>
+    <sheet name="Nota" sheetId="13" r:id="rId16"/>
+    <sheet name="Pajak_NTPN" sheetId="14" r:id="rId17"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
@@ -27,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="140">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="151">
   <si>
     <t>NAV</t>
   </si>
@@ -158,6 +159,42 @@
     <t>Honor Pengelola</t>
   </si>
   <si>
+    <t>kode</t>
+  </si>
+  <si>
+    <t>nama_sumber_dana</t>
+  </si>
+  <si>
+    <t>alias</t>
+  </si>
+  <si>
+    <t>is_sumber_dana_tambahan</t>
+  </si>
+  <si>
+    <t>is_afirmasi</t>
+  </si>
+  <si>
+    <t>4.3.1.01.</t>
+  </si>
+  <si>
+    <t>BOS Reguler</t>
+  </si>
+  <si>
+    <t>4.3.1.05.</t>
+  </si>
+  <si>
+    <t>Lainnya</t>
+  </si>
+  <si>
+    <t>4.3.1.1005</t>
+  </si>
+  <si>
+    <t>Banpem Keterampilan Menulis pada Sekolah Dasar</t>
+  </si>
+  <si>
+    <t>Banpem Keterampilan Menulis</t>
+  </si>
+  <si>
     <t>tanggal_aktivasi</t>
   </si>
   <si>
@@ -210,9 +247,6 @@
   </si>
   <si>
     <t>paket</t>
-  </si>
-  <si>
-    <t>BOS Reguler</t>
   </si>
   <si>
     <t>RAPBS-2</t>
@@ -834,33 +868,53 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>64</v>
       </c>
       <c r="B2" t="s">
-        <v>51</v>
+        <v>77</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3">
+        <v>78</v>
+      </c>
+      <c r="D2" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>58</v>
-      </c>
-      <c r="C3">
+        <v>81</v>
+      </c>
+      <c r="C3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" t="s">
+        <v>83</v>
+      </c>
+      <c r="C4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D4">
         <v>2</v>
       </c>
     </row>
@@ -876,362 +930,34 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:W11"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="C2" t="s">
-        <v>53</v>
-      </c>
-      <c r="D2" t="s">
-        <v>37</v>
-      </c>
-      <c r="E2" t="s">
-        <v>78</v>
-      </c>
-      <c r="F2" t="s">
-        <v>79</v>
-      </c>
-      <c r="G2" t="s">
-        <v>80</v>
-      </c>
-      <c r="H2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I2" t="s">
-        <v>54</v>
-      </c>
-      <c r="J2" t="s">
-        <v>82</v>
-      </c>
-      <c r="K2" t="s">
-        <v>83</v>
-      </c>
-      <c r="L2" t="s">
-        <v>84</v>
-      </c>
-      <c r="M2" t="s">
-        <v>85</v>
-      </c>
-      <c r="N2" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>86</v>
       </c>
-      <c r="O2" t="s">
-        <v>87</v>
-      </c>
-      <c r="P2" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q2" t="s">
-        <v>14</v>
-      </c>
-      <c r="R2" t="s">
-        <v>57</v>
-      </c>
-      <c r="S2" t="s">
-        <v>9</v>
-      </c>
-      <c r="T2" t="s">
-        <v>15</v>
-      </c>
-      <c r="U2" t="s">
-        <v>89</v>
-      </c>
-      <c r="V2" t="s">
-        <v>74</v>
-      </c>
-      <c r="W2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="3" spans="1:23">
-      <c r="A3" t="s">
-        <v>91</v>
-      </c>
       <c r="B3" t="s">
-        <v>92</v>
-      </c>
-      <c r="C3" t="s">
-        <v>93</v>
-      </c>
-      <c r="E3" t="s">
-        <v>94</v>
-      </c>
-      <c r="F3" t="s">
-        <v>95</v>
-      </c>
-      <c r="G3">
-        <v>100000000</v>
-      </c>
-      <c r="Q3">
-        <v>2025</v>
-      </c>
-      <c r="R3" t="s">
-        <v>61</v>
-      </c>
-      <c r="S3" t="s">
-        <v>96</v>
-      </c>
-      <c r="U3" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="4" spans="1:23">
-      <c r="A4" t="s">
-        <v>98</v>
-      </c>
-      <c r="B4" t="s">
-        <v>99</v>
-      </c>
-      <c r="C4" t="s">
-        <v>100</v>
-      </c>
-      <c r="D4" t="s">
-        <v>41</v>
-      </c>
-      <c r="E4" t="s">
-        <v>101</v>
-      </c>
-      <c r="F4" t="s">
-        <v>102</v>
-      </c>
-      <c r="G4">
-        <v>5000000</v>
-      </c>
-      <c r="I4">
-        <v>5</v>
-      </c>
-      <c r="Q4">
-        <v>2025</v>
-      </c>
-      <c r="R4" t="s">
-        <v>61</v>
-      </c>
-      <c r="S4" t="s">
-        <v>96</v>
-      </c>
-      <c r="V4" t="s">
-        <v>75</v>
-      </c>
-      <c r="W4" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23">
-      <c r="A5" t="s">
-        <v>104</v>
-      </c>
-      <c r="B5" t="s">
-        <v>105</v>
-      </c>
-      <c r="C5" t="s">
-        <v>106</v>
-      </c>
-      <c r="D5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" t="s">
-        <v>101</v>
-      </c>
-      <c r="F5" t="s">
-        <v>102</v>
-      </c>
-      <c r="G5">
-        <v>2000000</v>
-      </c>
-      <c r="Q5">
-        <v>2025</v>
-      </c>
-      <c r="R5" t="s">
-        <v>61</v>
-      </c>
-      <c r="S5" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23">
-      <c r="A6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D6" t="s">
-        <v>41</v>
-      </c>
-      <c r="E6" t="s">
-        <v>108</v>
-      </c>
-      <c r="F6" t="s">
-        <v>109</v>
-      </c>
-      <c r="G6">
-        <v>100000</v>
-      </c>
-      <c r="K6">
-        <v>1</v>
-      </c>
-      <c r="Q6">
-        <v>2025</v>
-      </c>
-      <c r="R6" t="s">
-        <v>61</v>
-      </c>
-      <c r="S6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23">
-      <c r="A7" t="s">
-        <v>110</v>
-      </c>
-      <c r="C7" t="s">
-        <v>111</v>
-      </c>
-      <c r="D7" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" t="s">
-        <v>112</v>
-      </c>
-      <c r="F7" t="s">
-        <v>113</v>
-      </c>
-      <c r="G7">
-        <v>100000</v>
-      </c>
-      <c r="K7">
-        <v>1</v>
-      </c>
-      <c r="Q7">
-        <v>2025</v>
-      </c>
-      <c r="R7" t="s">
-        <v>61</v>
-      </c>
-      <c r="S7" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23">
-      <c r="A8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C8" t="s">
-        <v>115</v>
-      </c>
-      <c r="E8" t="s">
-        <v>115</v>
-      </c>
-      <c r="F8" t="s">
-        <v>95</v>
-      </c>
-      <c r="G8">
-        <v>10000000</v>
-      </c>
-      <c r="Q8">
-        <v>2025</v>
-      </c>
-      <c r="R8" t="s">
-        <v>61</v>
-      </c>
-      <c r="S8" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23">
-      <c r="A9" t="s">
-        <v>114</v>
-      </c>
-      <c r="C9" t="s">
-        <v>116</v>
-      </c>
-      <c r="E9" t="s">
-        <v>117</v>
-      </c>
-      <c r="F9" t="s">
-        <v>113</v>
-      </c>
-      <c r="G9">
-        <v>10000000</v>
-      </c>
-      <c r="Q9">
-        <v>2025</v>
-      </c>
-      <c r="R9" t="s">
-        <v>61</v>
-      </c>
-      <c r="S9" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
-      <c r="A10" t="s">
-        <v>18</v>
-      </c>
-      <c r="C10" t="s">
-        <v>118</v>
-      </c>
-      <c r="E10" t="s">
-        <v>119</v>
-      </c>
-      <c r="F10" t="s">
-        <v>120</v>
-      </c>
-      <c r="Q10">
-        <v>2025</v>
-      </c>
-      <c r="R10" t="s">
-        <v>61</v>
-      </c>
-      <c r="S10" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23">
-      <c r="A11" t="s">
-        <v>121</v>
-      </c>
-      <c r="B11" t="s">
-        <v>122</v>
-      </c>
-      <c r="C11" t="s">
-        <v>123</v>
-      </c>
-      <c r="D11" t="s">
-        <v>41</v>
-      </c>
-      <c r="E11" t="s">
-        <v>101</v>
-      </c>
-      <c r="F11" t="s">
-        <v>102</v>
-      </c>
-      <c r="G11">
-        <v>999000</v>
-      </c>
-      <c r="Q11">
-        <v>2025</v>
-      </c>
-      <c r="R11" t="s">
-        <v>61</v>
-      </c>
-      <c r="S11" t="s">
-        <v>96</v>
-      </c>
-      <c r="T11">
-        <v>1</v>
+        <v>70</v>
+      </c>
+      <c r="C3">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -1246,90 +972,361 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:W11"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:23">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:23">
       <c r="A2" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" t="s">
+        <v>65</v>
+      </c>
+      <c r="D2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F2" t="s">
         <v>90</v>
       </c>
-      <c r="B2" t="s">
-        <v>77</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="G2" t="s">
+        <v>91</v>
+      </c>
+      <c r="H2" t="s">
+        <v>92</v>
+      </c>
+      <c r="I2" t="s">
+        <v>66</v>
+      </c>
+      <c r="J2" t="s">
+        <v>93</v>
+      </c>
+      <c r="K2" t="s">
+        <v>94</v>
+      </c>
+      <c r="L2" t="s">
+        <v>95</v>
+      </c>
+      <c r="M2" t="s">
+        <v>96</v>
+      </c>
+      <c r="N2" t="s">
+        <v>97</v>
+      </c>
+      <c r="O2" t="s">
+        <v>98</v>
+      </c>
+      <c r="P2" t="s">
+        <v>99</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>14</v>
+      </c>
+      <c r="R2" t="s">
+        <v>69</v>
+      </c>
+      <c r="S2" t="s">
+        <v>9</v>
+      </c>
+      <c r="T2" t="s">
+        <v>15</v>
+      </c>
+      <c r="U2" t="s">
+        <v>100</v>
+      </c>
+      <c r="V2" t="s">
+        <v>85</v>
+      </c>
+      <c r="W2" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
+      <c r="A3" t="s">
+        <v>102</v>
+      </c>
+      <c r="B3" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E3" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" t="s">
+        <v>106</v>
+      </c>
+      <c r="G3">
+        <v>100000000</v>
+      </c>
+      <c r="Q3">
+        <v>2025</v>
+      </c>
+      <c r="R3" t="s">
+        <v>49</v>
+      </c>
+      <c r="S3" t="s">
+        <v>107</v>
+      </c>
+      <c r="U3" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
+      <c r="A4" t="s">
+        <v>109</v>
+      </c>
+      <c r="B4" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" t="s">
+        <v>111</v>
+      </c>
+      <c r="D4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E4" t="s">
+        <v>112</v>
+      </c>
+      <c r="F4" t="s">
+        <v>113</v>
+      </c>
+      <c r="G4">
+        <v>5000000</v>
+      </c>
+      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="Q4">
+        <v>2025</v>
+      </c>
+      <c r="R4" t="s">
+        <v>49</v>
+      </c>
+      <c r="S4" t="s">
+        <v>107</v>
+      </c>
+      <c r="V4" t="s">
+        <v>86</v>
+      </c>
+      <c r="W4" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
+      <c r="A5" t="s">
+        <v>115</v>
+      </c>
+      <c r="B5" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
+        <v>112</v>
+      </c>
+      <c r="F5" t="s">
+        <v>113</v>
+      </c>
+      <c r="G5">
+        <v>2000000</v>
+      </c>
+      <c r="Q5">
+        <v>2025</v>
+      </c>
+      <c r="R5" t="s">
+        <v>49</v>
+      </c>
+      <c r="S5" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
+      <c r="A6" t="s">
+        <v>109</v>
+      </c>
+      <c r="C6" t="s">
+        <v>118</v>
+      </c>
+      <c r="D6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F6" t="s">
+        <v>120</v>
+      </c>
+      <c r="G6">
+        <v>100000</v>
+      </c>
+      <c r="K6">
+        <v>1</v>
+      </c>
+      <c r="Q6">
+        <v>2025</v>
+      </c>
+      <c r="R6" t="s">
+        <v>49</v>
+      </c>
+      <c r="S6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23">
+      <c r="A7" t="s">
+        <v>121</v>
+      </c>
+      <c r="C7" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E7" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" t="s">
         <v>124</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G7">
+        <v>100000</v>
+      </c>
+      <c r="K7">
+        <v>1</v>
+      </c>
+      <c r="Q7">
+        <v>2025</v>
+      </c>
+      <c r="R7" t="s">
+        <v>49</v>
+      </c>
+      <c r="S7" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23">
+      <c r="A8" t="s">
         <v>125</v>
       </c>
-      <c r="E2" t="s">
+      <c r="C8" t="s">
         <v>126</v>
       </c>
-      <c r="F2" t="s">
+      <c r="E8" t="s">
+        <v>126</v>
+      </c>
+      <c r="F8" t="s">
+        <v>106</v>
+      </c>
+      <c r="G8">
+        <v>10000000</v>
+      </c>
+      <c r="Q8">
+        <v>2025</v>
+      </c>
+      <c r="R8" t="s">
+        <v>49</v>
+      </c>
+      <c r="S8" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23">
+      <c r="A9" t="s">
+        <v>125</v>
+      </c>
+      <c r="C9" t="s">
         <v>127</v>
       </c>
-      <c r="G2" t="s">
+      <c r="E9" t="s">
         <v>128</v>
       </c>
-      <c r="H2" t="s">
+      <c r="F9" t="s">
+        <v>124</v>
+      </c>
+      <c r="G9">
+        <v>10000000</v>
+      </c>
+      <c r="Q9">
+        <v>2025</v>
+      </c>
+      <c r="R9" t="s">
+        <v>49</v>
+      </c>
+      <c r="S9" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23">
+      <c r="A10" t="s">
+        <v>18</v>
+      </c>
+      <c r="C10" t="s">
         <v>129</v>
       </c>
-      <c r="I2" t="s">
+      <c r="E10" t="s">
         <v>130</v>
       </c>
-      <c r="J2" t="s">
-        <v>37</v>
-      </c>
-      <c r="K2" t="s">
+      <c r="F10" t="s">
         <v>131</v>
       </c>
-      <c r="L2" t="s">
+      <c r="Q10">
+        <v>2025</v>
+      </c>
+      <c r="R10" t="s">
+        <v>49</v>
+      </c>
+      <c r="S10" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23">
+      <c r="A11" t="s">
         <v>132</v>
       </c>
-      <c r="M2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N2" t="s">
+      <c r="B11" t="s">
         <v>133</v>
       </c>
-    </row>
-    <row r="3" spans="1:14">
-      <c r="A3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B3" t="s">
-        <v>99</v>
-      </c>
-      <c r="C3" t="s">
-        <v>98</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C11" t="s">
         <v>134</v>
       </c>
-      <c r="E3" t="s">
-        <v>135</v>
-      </c>
-      <c r="F3" t="s">
-        <v>136</v>
-      </c>
-      <c r="G3" t="s">
-        <v>137</v>
-      </c>
-      <c r="H3">
-        <v>123456789012345</v>
-      </c>
-      <c r="I3">
-        <v>5000000</v>
-      </c>
-      <c r="J3" t="s">
+      <c r="D11" t="s">
         <v>41</v>
       </c>
-      <c r="N3">
+      <c r="E11" t="s">
+        <v>112</v>
+      </c>
+      <c r="F11" t="s">
+        <v>113</v>
+      </c>
+      <c r="G11">
+        <v>999000</v>
+      </c>
+      <c r="Q11">
+        <v>2025</v>
+      </c>
+      <c r="R11" t="s">
+        <v>49</v>
+      </c>
+      <c r="S11" t="s">
+        <v>107</v>
+      </c>
+      <c r="T11">
         <v>1</v>
       </c>
     </row>
@@ -1345,6 +1342,105 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" spans="1:14">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" t="s">
+        <v>88</v>
+      </c>
+      <c r="C2" t="s">
+        <v>135</v>
+      </c>
+      <c r="D2" t="s">
+        <v>136</v>
+      </c>
+      <c r="E2" t="s">
+        <v>137</v>
+      </c>
+      <c r="F2" t="s">
+        <v>138</v>
+      </c>
+      <c r="G2" t="s">
+        <v>139</v>
+      </c>
+      <c r="H2" t="s">
+        <v>140</v>
+      </c>
+      <c r="I2" t="s">
+        <v>141</v>
+      </c>
+      <c r="J2" t="s">
+        <v>37</v>
+      </c>
+      <c r="K2" t="s">
+        <v>142</v>
+      </c>
+      <c r="L2" t="s">
+        <v>143</v>
+      </c>
+      <c r="M2" t="s">
+        <v>15</v>
+      </c>
+      <c r="N2" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" t="s">
+        <v>114</v>
+      </c>
+      <c r="B3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C3" t="s">
+        <v>109</v>
+      </c>
+      <c r="D3" t="s">
+        <v>145</v>
+      </c>
+      <c r="E3" t="s">
+        <v>146</v>
+      </c>
+      <c r="F3" t="s">
+        <v>147</v>
+      </c>
+      <c r="G3" t="s">
+        <v>148</v>
+      </c>
+      <c r="H3">
+        <v>123456789012345</v>
+      </c>
+      <c r="I3">
+        <v>5000000</v>
+      </c>
+      <c r="J3" t="s">
+        <v>41</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
   <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
@@ -1355,10 +1451,10 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="C2" t="s">
         <v>15</v>
@@ -1366,10 +1462,10 @@
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="B3" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
     </row>
   </sheetData>
@@ -1643,37 +1739,71 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
         <v>43</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>44</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>45</v>
       </c>
-      <c r="D2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4">
-      <c r="A3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3">
-        <v>500000</v>
-      </c>
-      <c r="C3">
-        <v>250000</v>
+      <c r="E2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>1</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>5</v>
+      </c>
+      <c r="B4" t="s">
+        <v>50</v>
+      </c>
+      <c r="C4" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>1005</v>
+      </c>
+      <c r="B5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" t="s">
+        <v>53</v>
+      </c>
+      <c r="D5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -1688,39 +1818,37 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>46</v>
+        <v>55</v>
       </c>
       <c r="B2" t="s">
-        <v>2</v>
+        <v>56</v>
       </c>
       <c r="C2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D2" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>47</v>
-      </c>
-      <c r="B3" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" t="s">
-        <v>49</v>
-      </c>
-      <c r="B4" t="s">
-        <v>50</v>
+        <v>18</v>
+      </c>
+      <c r="B3">
+        <v>500000</v>
+      </c>
+      <c r="C3">
+        <v>250000</v>
       </c>
     </row>
   </sheetData>
@@ -1735,140 +1863,39 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>52</v>
+        <v>2</v>
       </c>
       <c r="C2" t="s">
-        <v>37</v>
-      </c>
-      <c r="D2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G2" t="s">
-        <v>56</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" t="s">
         <v>15</v>
       </c>
-      <c r="J2" t="s">
-        <v>14</v>
-      </c>
-      <c r="K2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11">
+    </row>
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
-      </c>
-      <c r="C3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
         <v>60</v>
       </c>
-      <c r="G3">
-        <v>500000</v>
-      </c>
-      <c r="H3">
-        <v>1000000</v>
-      </c>
-      <c r="J3">
-        <v>2025</v>
-      </c>
-      <c r="K3" t="s">
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="4" spans="1:11">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>62</v>
-      </c>
-      <c r="C4" t="s">
-        <v>39</v>
-      </c>
-      <c r="D4" t="s">
-        <v>63</v>
-      </c>
-      <c r="E4">
-        <v>1</v>
-      </c>
-      <c r="F4" t="s">
-        <v>60</v>
-      </c>
-      <c r="G4">
-        <v>100000</v>
-      </c>
-      <c r="H4">
-        <v>100000</v>
-      </c>
-      <c r="J4">
-        <v>2025</v>
-      </c>
-      <c r="K4" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11">
-      <c r="A5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C5" t="s">
-        <v>41</v>
-      </c>
-      <c r="D5" t="s">
-        <v>65</v>
-      </c>
-      <c r="E5">
-        <v>1</v>
-      </c>
-      <c r="F5" t="s">
-        <v>60</v>
-      </c>
-      <c r="G5">
-        <v>50000</v>
-      </c>
-      <c r="H5">
-        <v>50000</v>
-      </c>
-      <c r="I5">
-        <v>1</v>
-      </c>
-      <c r="J5">
-        <v>2025</v>
-      </c>
-      <c r="K5" t="s">
-        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -1883,54 +1910,140 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:11">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
+    <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>52</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
+        <v>64</v>
+      </c>
+      <c r="C2" t="s">
+        <v>37</v>
+      </c>
+      <c r="D2" t="s">
+        <v>65</v>
+      </c>
+      <c r="E2" t="s">
         <v>66</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F2" t="s">
         <v>67</v>
       </c>
-      <c r="D2" t="s">
+      <c r="G2" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="3" spans="1:4">
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J2" t="s">
+        <v>14</v>
+      </c>
+      <c r="K2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11">
       <c r="A3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C3" t="s">
-        <v>71</v>
-      </c>
-      <c r="D3">
+        <v>41</v>
+      </c>
+      <c r="D3" t="s">
+        <v>42</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3">
+        <v>500000</v>
+      </c>
+      <c r="H3">
+        <v>1000000</v>
+      </c>
+      <c r="J3">
+        <v>2025</v>
+      </c>
+      <c r="K3" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11">
+      <c r="A4" t="s">
+        <v>73</v>
+      </c>
+      <c r="C4" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4">
         <v>1</v>
       </c>
-    </row>
-    <row r="4" spans="1:4">
-      <c r="A4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="F4" t="s">
         <v>72</v>
       </c>
-      <c r="C4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4">
-        <v>2</v>
+      <c r="G4">
+        <v>100000</v>
+      </c>
+      <c r="H4">
+        <v>100000</v>
+      </c>
+      <c r="J4">
+        <v>2025</v>
+      </c>
+      <c r="K4" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11">
+      <c r="A5" t="s">
+        <v>75</v>
+      </c>
+      <c r="C5" t="s">
+        <v>41</v>
+      </c>
+      <c r="D5" t="s">
+        <v>76</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5" t="s">
+        <v>72</v>
+      </c>
+      <c r="G5">
+        <v>50000</v>
+      </c>
+      <c r="H5">
+        <v>50000</v>
+      </c>
+      <c r="I5">
+        <v>1</v>
+      </c>
+      <c r="J5">
+        <v>2025</v>
+      </c>
+      <c r="K5" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>